<commit_message>
test: record final S01-B runtime recovery and acceptance evidence
</commit_message>
<xml_diff>
--- a/evidence/pg16_normal_sample_1.xlsx
+++ b/evidence/pg16_normal_sample_1.xlsx
@@ -87,7 +87,7 @@
     <t>snapshot_id</t>
   </si>
   <si>
-    <t>1b7c35ba55dfefd3dbd71d2610b2db80</t>
+    <t>546e915b6bd7375d199d225510262fd6</t>
   </si>
   <si>
     <t>integration_id</t>
@@ -129,13 +129,13 @@
     <t>source_snapshot_ref</t>
   </si>
   <si>
-    <t>7df1da6af74ac1a76adda3f60e4ed0d9</t>
+    <t>ca12304cbdf899f8df484c5343bb23ee</t>
   </si>
   <si>
     <t>expires_at</t>
   </si>
   <si>
-    <t>2026-10-26T07:04:54Z</t>
+    <t>2026-10-26T07:29:01Z</t>
   </si>
   <si>
     <t>precision</t>

</xml_diff>